<commit_message>
Added new RDF data schemes and visual schemes for employment-table16-20, fixed XLSX spreadsheets for employment-table16-20
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/employment-table16.xlsx
+++ b/sources/table_normalization/xlsx/employment-table16.xlsx
@@ -158,16 +158,16 @@
   </cellStyleXfs>
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -477,115 +477,115 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5">
+      <c r="B1" s="3">
         <v>2023</v>
       </c>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="5"/>
-      <c r="I1" s="5"/>
-      <c r="J1" s="5"/>
-      <c r="K1" s="5"/>
-      <c r="L1" s="5"/>
-      <c r="M1" s="5"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="L1" s="3"/>
+      <c r="M1" s="3"/>
     </row>
     <row r="2" spans="1:13">
-      <c r="A2" s="3"/>
-      <c r="B2" s="6" t="s">
+      <c r="A2" s="2"/>
+      <c r="B2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6" t="s">
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6"/>
-      <c r="J2" s="6"/>
-      <c r="K2" s="6"/>
-      <c r="L2" s="6"/>
-      <c r="M2" s="6"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
     </row>
     <row r="3" spans="1:13">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3" t="s">
+      <c r="A3" s="2"/>
+      <c r="B3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
-      <c r="J3" s="3"/>
-      <c r="K3" s="3"/>
-      <c r="L3" s="4" t="s">
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="M3" s="4" t="s">
+      <c r="M3" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:13">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3" t="s">
+      <c r="A4" s="2"/>
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="4" t="s">
+      <c r="I4" s="4"/>
+      <c r="J4" s="4"/>
+      <c r="K4" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="L4" s="3"/>
-      <c r="M4" s="3"/>
+      <c r="L4" s="4"/>
+      <c r="M4" s="4"/>
     </row>
     <row r="5" spans="1:13" ht="51.5" customHeight="1">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
+      <c r="A5" s="2"/>
+      <c r="B5" s="4"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4"/>
       <c r="H5" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="I5" s="2" t="s">
+      <c r="I5" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="J5" s="2" t="s">
+      <c r="J5" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K5" s="3"/>
-      <c r="L5" s="3"/>
-      <c r="M5" s="3"/>
+      <c r="K5" s="4"/>
+      <c r="L5" s="4"/>
+      <c r="M5" s="4"/>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" t="s">

</xml_diff>